<commit_message>
v1.108: complete the log - previews gain a log writer, mains rows land within 250 ms, refresh state workbooks
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Documentation/System_State_Scenarios.xlsx
+++ b/Documentation/System_State_Scenarios.xlsx
@@ -1,108 +1,65 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="24000" windowHeight="12000" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="راهنما" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="States" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Transitions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Requirements" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Test_Cases" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Coverage" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Signals" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Faults" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Change_Log" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="راهنما" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="States" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transitions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test_Cases" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Signals" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Faults" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_Log" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'راهنما'!$A$3:$B$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'States'!$A$3:$G$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Transitions'!$A$3:$H$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Requirements'!$A$3:$F$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Test_Cases'!$A$3:$J$32</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Coverage'!$A$3:$E$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Signals'!$A$3:$F$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Faults'!$A$3:$F$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Change_Log'!$A$3:$E$5</definedName>
-  </definedNames>
-  <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
-    <font>
-      <name val="Aptos"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Aptos"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Aptos"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="12"/>
-    </font>
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
-      <sz val="12"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Vazirmatn"/>
+      <name val="B Nazanin"/>
       <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="12"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
     </font>
     <font>
-      <name val="Vazirmatn"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Vazirmatn"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Vazirmatn"/>
+      <name val="B Nazanin"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Vazirmatn"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="14"/>
+      <name val="B Nazanin"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="B Nazanin"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9EAF7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -114,8 +71,23 @@
         <fgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E2F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -124,73 +96,46 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin"/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal/>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+  <cellXfs count="7">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -552,3078 +497,3242 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" style="4" min="1" max="1"/>
-    <col width="100" customWidth="1" style="4" min="2" max="2"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="2" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" s="4">
-      <c r="A1" s="7" t="inlineStr">
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>راهنمای استفاده از مرجع State و Scenario</t>
         </is>
       </c>
-      <c r="B1" s="5" t="n"/>
-    </row>
-    <row r="2" ht="42" customHeight="1" s="4">
-      <c r="A2" s="8" t="inlineStr">
-        <is>
-          <t>این فایل مرجع سطح‌بالای State و سناریوهاست؛ جزئیات اندازه‌گیری را در Workbookهای ماژول ثبت کن.</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="n"/>
-    </row>
-    <row r="3" ht="42" customHeight="1" s="4">
-      <c r="A3" s="9" t="inlineStr">
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>موضوع</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>توضیح</t>
         </is>
       </c>
-    </row>
-    <row r="4" ht="32" customHeight="1" s="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>راهنمای استفاده</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>این Workbook مرجع سطح‌بالای State و سناریوهای سیستم ChangeOver است. جزئیات اجرایی هر ماژول در Workbookهای Validation همان ماژول ثبت می‌شود.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="32" customHeight="1" s="4">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>روش کار 1</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>روش کار ۱</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>ابتدا States و Transitions را بخوان؛ این دو برگه می‌گویند سیستم در هر شرط به کجا می‌رود.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="32" customHeight="1" s="4">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>روش کار 2</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>تست‌های ماژول‌ها در فایل ولیدیشن خودشان است (Firmware/Modules/&lt;Module&gt;) و اینجا تکرار نمی‌شود؛ در Test_Cases فقط تست‌های سطح سیستم (SYS/BZ/SAFE) اجرا و نتیجهٔ واقعی ثبت می‌شود.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="32" customHeight="1" s="4">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>روش کار 3</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>در Coverage مطمئن شو هر الزام حداقل یک تست دارد؛ وضعیت GAP نباید بدون توضیح باقی بماند.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="32" customHeight="1" s="4">
-      <c r="A8" s="8" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>روش کار ۲</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>تست‌های ماژول‌ها در فایل ولیدیشن خودشان است (Firmware/Modules/&lt;Module&gt;) و اینجا تکرار نمی‌شود؛ در Test_Cases فقط تست‌های سطح سیستم (SYS/BZ/SAFE) هستند.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>روش کار ۳</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>در Coverage مطمئن شو هر الزام حداقل یک تست دارد؛ وضعیت GAP نباید بدون توضیح بماند.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>اصل مهم</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>snapshot نامعتبر قبل از هر تصمیم state، fault، timer یا pin بررسی می‌شود.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="32" customHeight="1" s="4">
-      <c r="A9" s="8" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Build فعلی</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>MODULE_UI=1، MODULE_MEASUREMENT=1، MODULE_CHANGEOVER=1، MODULE_FAULT=1، MODULE_CHARGER=1 (CHG_MASTER_ENABLE=1، CHG_TRANSFORMER_KNOWN=1)، MODULE_JITTER=1، MODULE_MCU_POWER_PATH=1؛ Protection و ESP فعلاً خاموش (وضعیت 2026-09-22).</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="32" customHeight="1" s="4">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>MODULE_UI=1، MODULE_MEASUREMENT=1، MODULE_CHANGEOVER=1، MODULE_FAULT=1، MODULE_CHARGER=1 (CHG_MASTER_ENABLE=1، CHG_TRANSFORMER_KNOWN=1)، MODULE_IMBALANCE=1، MODULE_ESPLINK=1، MODULE_JITTER=1، MODULE_PROTECTION=0، MODULE_MCU_POWER_PATH=1، MODULE_DIAG=1، MODULE_FLASH_LOCK=1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>محدودیت تست</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>تست Host و syntax جای تست واقعی برد نیستند. برای Fault با Protection خاموش، fault باید از مسیر تست تزریق شود.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="32" customHeight="1" s="4">
-      <c r="A11" s="8" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>فایل‌های جزئیات</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>UI_Board_Validation.xlsx، Buzzer_Board_Validation.xlsx، Measurement_Board_Validation.xlsx و Changeover_Board_Validation.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="32" customHeight="1" s="4">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>UI_Board_Validation.xlsx، Measurement_Board_Validation.xlsx، Changeover_Board_Validation.xlsx و بقیهٔ Workbookهای ماژول‌ها.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>تعریف PASS</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>فقط وقتی PASS ثبت شود که نتیجه واقعی با معیار قبولی ردیف منطبق باشد و مدرک تست ثبت شده باشد.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="32" customHeight="1" s="4">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>فقط وقتی PASS ثبت شود که نتیجهٔ واقعی با معیار قبولی ردیف منطبق باشد و مدرک تست ثبت شده باشد.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>تازه‌سازی</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>این فایل با کد تولید می‌شود؛ دستی ویرایش نکن. دستور: python3 tools/make_state_reference_xlsx.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>تاریخ تهیه</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-16 | بازسازی از کد فعلی: 2026-10-24</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:B13"/>
-  <mergeCells count="2">
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A1:B1"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
   </mergeCells>
-  <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="007030A0"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" style="4" min="1" max="1"/>
-    <col width="32" customWidth="1" style="4" min="2" max="2"/>
-    <col width="24" customWidth="1" style="4" min="3" max="3"/>
-    <col width="42" customWidth="1" style="4" min="4" max="4"/>
-    <col width="42" customWidth="1" style="4" min="5" max="5"/>
-    <col width="40" customWidth="1" style="4" min="6" max="6"/>
-    <col width="24" customWidth="1" style="4" min="7" max="7"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" s="4">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>States — حالت‌های رسمی سیستم</t>
-        </is>
-      </c>
-      <c r="B1" s="6" t="n"/>
-      <c r="C1" s="6" t="n"/>
-      <c r="D1" s="6" t="n"/>
-      <c r="E1" s="6" t="n"/>
-      <c r="F1" s="6" t="n"/>
-      <c r="G1" s="5" t="n"/>
-    </row>
-    <row r="2" ht="42" customHeight="1" s="4">
-      <c r="A2" s="8" t="inlineStr">
-        <is>
-          <t>هر ردیف یک حالت رسمی سیستم است. خروجی امن و تست‌های مرجع را از همین جدول بخوان.</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="n"/>
-      <c r="C2" s="6" t="n"/>
-      <c r="D2" s="6" t="n"/>
-      <c r="E2" s="6" t="n"/>
-      <c r="F2" s="6" t="n"/>
-      <c r="G2" s="5" t="n"/>
-    </row>
-    <row r="3" ht="42" customHeight="1" s="4">
-      <c r="A3" s="9" t="inlineStr">
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>States — حالت‌های رسمی سیستم (Changeover + UI)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>معنی</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>ورودی معتبر لازم</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>خروجی/رفتار مورد انتظار</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>شرط خروج</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
-        <is>
-          <t>Safe behavior</t>
-        </is>
-      </c>
-      <c r="G3" s="9" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>تست مرجع</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="54" customHeight="1" s="4">
-      <c r="A4" s="8" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>BOOT</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>شروع یا مقداردهی اولیه</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>خیر/هنوز snapshot معتبر نیست</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
-        <is>
-          <t>state اولیه؛ PB11 از BSP در حالت Safe High</t>
-        </is>
-      </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>state اولیه؛ PB11 در حالت Safe High</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>snapshot معتبر و input_present یا fault</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t>invalid: حفظ BOOT و PB11</t>
-        </is>
-      </c>
-      <c r="G4" s="8" t="inlineStr">
-        <is>
-          <t>CO-001, CO-003</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="54" customHeight="1" s="4">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>BATTERY</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>ورودی اصلی حاضر نیست و مسیر باتری برقرار است</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>بله، valid=true و input_present=false</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>PB11 High؛ UI در BatteryRun</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>cut condition یا input_present=true</t>
         </is>
       </c>
-      <c r="F5" s="8" t="inlineStr">
-        <is>
-          <t>fault معتبر: FAULT بدون تغییر pin</t>
-        </is>
-      </c>
-      <c r="G5" s="8" t="inlineStr">
-        <is>
-          <t>CO-006, UI-008</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="54" customHeight="1" s="4">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>CO-006</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>INPUT</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>ورودی اصلی حاضر است</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>بله، valid=true و input_present=true</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>PB11 High؛ UI در InputOk/Charging</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>cut condition یا input_present=false</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>fault معتبر: FAULT بدون تغییر pin</t>
-        </is>
-      </c>
-      <c r="G6" s="8" t="inlineStr">
-        <is>
-          <t>CO-007, UI-003</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="54" customHeight="1" s="4">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>CO-007</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>SAFE</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>مسیر باتری قطع شده است</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>بله برای ورود؛ در invalid حفظ می‌شود</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>PB11 Low؛ تا reconnect قطع باقی می‌ماند</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
-        <is>
-          <t>input_present=true و v_bat24_mv&gt;=21200 برای 3000ms</t>
-        </is>
-      </c>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>invalid/fault: حفظ SAFE و PB11 Low</t>
-        </is>
-      </c>
-      <c r="G7" s="8" t="inlineStr">
-        <is>
-          <t>CO-008, CO-013, CO-017, CO-018</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="54" customHeight="1" s="4">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>input_present=true و v_bat24≥21200 (یا بازیابی بدون برق شهر — ST-011)</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>CO-013..016</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>FAULT</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>fault معتبر در snapshot معتبر</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>snapshot.valid=true و fault_mask!=0</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>state=FAULT؛ هیچ pin توسط Fault تغییر نمی‌کند</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>fault پاک شود و منطق valid دوباره ارزیابی شود</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>invalid: اصلاً وارد FAULT نشود</t>
-        </is>
-      </c>
-      <c r="G8" s="8" t="inlineStr">
-        <is>
-          <t>CO-003, CO-004, CO-005</t>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>fault پاک شود</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>CO-004, CO-005</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:G8"/>
-  <mergeCells count="2">
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="007030A0"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" style="4" min="1" max="1"/>
-    <col width="20" customWidth="1" style="4" min="2" max="2"/>
-    <col width="56" customWidth="1" style="4" min="3" max="3"/>
-    <col width="18" customWidth="1" style="4" min="4" max="4"/>
-    <col width="48" customWidth="1" style="4" min="5" max="5"/>
-    <col width="20" customWidth="1" style="4" min="6" max="6"/>
-    <col width="24" customWidth="1" style="4" min="7" max="7"/>
-    <col width="36" customWidth="1" style="4" min="8" max="8"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" s="4">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>Transitions — مسیرهای تغییر حالت</t>
-        </is>
-      </c>
-      <c r="B1" s="6" t="n"/>
-      <c r="C1" s="6" t="n"/>
-      <c r="D1" s="6" t="n"/>
-      <c r="E1" s="6" t="n"/>
-      <c r="F1" s="6" t="n"/>
-      <c r="G1" s="6" t="n"/>
-      <c r="H1" s="5" t="n"/>
-    </row>
-    <row r="2" ht="42" customHeight="1" s="4">
-      <c r="A2" s="8" t="inlineStr">
-        <is>
-          <t>هر ردیف یک transition مستقل است؛ شرط، زمان، اقدام و state مقصد باید با کد یکسان باشد.</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="n"/>
-      <c r="C2" s="6" t="n"/>
-      <c r="D2" s="6" t="n"/>
-      <c r="E2" s="6" t="n"/>
-      <c r="F2" s="6" t="n"/>
-      <c r="G2" s="6" t="n"/>
-      <c r="H2" s="5" t="n"/>
-    </row>
-    <row r="3" ht="42" customHeight="1" s="4">
-      <c r="A3" s="9" t="inlineStr">
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Transitions — مسیرهای تغییر حالت (اعداد از کد فعلی)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>From</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Trigger / guard</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Timer</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Action / output</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>To</t>
         </is>
       </c>
-      <c r="G3" s="9" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Validation</t>
         </is>
       </c>
-      <c r="H3" s="9" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>توضیح</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="54" customHeight="1" s="4">
-      <c r="A4" s="8" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>ST-001</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>هر state</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>snapshot=NULL یا valid=false</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>فوری</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>cut/reconnect timer reset؛ state و PB11 حفظ</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>همان state</t>
         </is>
       </c>
-      <c r="G4" s="8" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>CO-001, CO-002, CO-017</t>
         </is>
       </c>
-      <c r="H4" s="8" t="inlineStr">
-        <is>
-          <t>fault در این مسیر نباید FAULT بسازد</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="54" customHeight="1" s="4">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>invalid قبل از هر تصمیمی</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>ST-002</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>BOOT</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>valid=true و input_present=false</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>فوری</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>بدون cut؛ PB11 High</t>
         </is>
       </c>
-      <c r="F5" s="8" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>BATTERY</t>
         </is>
       </c>
-      <c r="G5" s="8" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>CO-006</t>
         </is>
       </c>
-      <c r="H5" s="8" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>mapping معتبر</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="54" customHeight="1" s="4">
-      <c r="A6" s="8" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>ST-003</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>BOOT</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>valid=true و input_present=true</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>فوری</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>بدون cut؛ PB11 High</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>INPUT</t>
         </is>
       </c>
-      <c r="G6" s="8" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>CO-007</t>
         </is>
       </c>
-      <c r="H6" s="8" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>mapping معتبر</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="54" customHeight="1" s="4">
-      <c r="A7" s="8" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>ST-004</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>BATTERY/INPUT</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>v_bat24_mv&lt;21000 و UI flag=true</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>v_bat24&lt;21000 و قفل باتری کم</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>3000ms پیوسته</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>BSP_GPIO_PROTECT_BATTERY=true</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>SAFE</t>
         </is>
       </c>
-      <c r="G7" s="8" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>CO-008</t>
         </is>
       </c>
-      <c r="H7" s="8" t="inlineStr">
-        <is>
-          <t>cut گیت‌شده؛ 21000 دقیق cut نیست</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="54" customHeight="1" s="4">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>cut گیت‌شده؛ ۲۱۰۰۰ دقیق</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>ST-005</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>BATTERY/INPUT</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>v_bat24_mv&lt;20800، مستقل از UI flag</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>v_bat24&lt;20800، مستقل از قفل</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>3000ms پیوسته</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>BSP_GPIO_PROTECT_BATTERY=true</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>SAFE</t>
         </is>
       </c>
-      <c r="G8" s="8" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>CO-009</t>
         </is>
       </c>
-      <c r="H8" s="8" t="inlineStr">
-        <is>
-          <t>cut مستقل؛ 20800 دقیق cut نیست</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="54" customHeight="1" s="4">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>cut مستقل؛ ۲۰۸۰۰ دقیق</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>ST-006</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>SAFE</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>input_present=true و v_bat24_mv&gt;=21200</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>3000ms پیوسته</t>
-        </is>
-      </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>input_present=true و v_bat24≥21200</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>30s پایداری ورودی + 3000ms ولتاژ</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>BSP_GPIO_PROTECT_BATTERY=false</t>
         </is>
       </c>
-      <c r="F9" s="8" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>INPUT</t>
         </is>
       </c>
-      <c r="G9" s="8" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>CO-013, CO-014</t>
         </is>
       </c>
-      <c r="H9" s="8" t="inlineStr">
-        <is>
-          <t>reconnect؛ 21200 شامل می‌شود</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="54" customHeight="1" s="4">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>بازگشت با برق شهر؛ ۲۱۲۰۰ آستانه</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>ST-007</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>هر state معتبر</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>snapshot.valid=true و fault_mask!=0</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>fault_mask!=0</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>فوری</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>state=FAULT؛ pin بدون تغییر</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>FAULT</t>
         </is>
       </c>
-      <c r="G10" s="8" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>CO-004, CO-005</t>
         </is>
       </c>
-      <c r="H10" s="8" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>fault اولویت دارد</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="54" customHeight="1" s="4">
-      <c r="A11" s="8" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>ST-008</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>هر state</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>snapshot.invalid و fault_mask!=0</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>فوری</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>fault نادیده؛ timer reset؛ pin حفظ</t>
         </is>
       </c>
-      <c r="F11" s="8" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>همان state</t>
         </is>
       </c>
-      <c r="G11" s="8" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>CO-003</t>
         </is>
       </c>
-      <c r="H11" s="8" t="inlineStr">
-        <is>
-          <t>invalid قبل از fault است</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="54" customHeight="1" s="4">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>invalid قبل از fault</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>ST-009</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>هر state معتبر</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>MillisecondsToTicks(3000)==0</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>فوری</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>هیچ cut/reconnect فوری؛ timer reset</t>
         </is>
       </c>
-      <c r="F12" s="8" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>همان state</t>
         </is>
       </c>
-      <c r="G12" s="8" t="inlineStr">
+      <c r="G11" s="4" t="inlineStr">
         <is>
           <t>CO-022</t>
         </is>
       </c>
-      <c r="H12" s="8" t="inlineStr">
-        <is>
-          <t>durationTicks صفر guard دارد</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="54" customHeight="1" s="4">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>guard صفر</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>ST-010</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>FAULT</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>valid=true و fault_mask=0</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>فوری</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>mapping عادی یا SAFE بر اساس protect</t>
         </is>
       </c>
-      <c r="F13" s="8" t="inlineStr">
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>INPUT/BATTERY/SAFE</t>
         </is>
       </c>
-      <c r="G13" s="8" t="inlineStr">
+      <c r="G12" s="5" t="inlineStr">
         <is>
           <t>CO-004 تکمیلی</t>
         </is>
       </c>
-      <c r="H13" s="8" t="inlineStr">
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>بسته به protect و input</t>
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>ST-011</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>SAFE (بدون برق شهر)</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>v_bat24≥21200 بی‌وقفه (۱۰s، هر افت = صفر) + فیلتر 3000ms</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>10000ms + 3000ms</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>مسیر باتری وصل می‌شود (یک تلاش)</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>BATTERY</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>CO-015/016</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>بازیابی بدون برق شهر (۲۰۲۶-۱۰-۲۳)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>ST-012</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>BATTERY (پس از ST-011)</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>قطع دوباره داخل ۶۰s</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>60000ms</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>حکم باتری ضعیف (سناریوی ۸) قفل می‌شود؛ مسیر بسته</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>SAFE + حکم ۸</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>محافظ چرخه؛ فقط برق شهر (۳۰s+3s) یا پاک‌کردن حکم باز می‌کند</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>ST-013</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>SAFE + حکم ۸</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>v_bat24≥21200 پیوسته ۱۰ دقیقه (یا «ریست قفل‌ها»)</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>600000ms</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>حکم پاک و یک تلاش مجدد</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>BATTERY</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>پاک‌شدن خودکار هشدار باتری فرسوده</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:H13"/>
-  <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
+  <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
-  <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00BF8F00"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" style="4" min="1" max="1"/>
-    <col width="16" customWidth="1" style="4" min="2" max="2"/>
-    <col width="74" customWidth="1" style="4" min="3" max="3"/>
-    <col width="34" customWidth="1" style="4" min="4" max="4"/>
-    <col width="30" customWidth="1" style="4" min="5" max="5"/>
-    <col width="18" customWidth="1" style="4" min="6" max="6"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="56" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" s="4">
-      <c r="A1" s="7" t="inlineStr">
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Requirements — الزامات قابل ردیابی</t>
         </is>
       </c>
-      <c r="B1" s="6" t="n"/>
-      <c r="C1" s="6" t="n"/>
-      <c r="D1" s="6" t="n"/>
-      <c r="E1" s="6" t="n"/>
-      <c r="F1" s="5" t="n"/>
-    </row>
-    <row r="2" ht="42" customHeight="1" s="4">
-      <c r="A2" s="8" t="inlineStr">
-        <is>
-          <t>هر الزام باید حداقل یک Test ID داشته باشد؛ وضعیت «در انتظار» یعنی هنوز روی برد اجرا نشده.</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="n"/>
-      <c r="C2" s="6" t="n"/>
-      <c r="D2" s="6" t="n"/>
-      <c r="E2" s="6" t="n"/>
-      <c r="F2" s="5" t="n"/>
-    </row>
-    <row r="3" ht="42" customHeight="1" s="4">
-      <c r="A3" s="9" t="inlineStr">
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Area</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Requirement دقیق</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>منبع/ثابت</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>تست پوشش‌دهنده</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>وضعیت</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="32" customHeight="1" s="4">
-      <c r="A4" s="8" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>REQ-M-001</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Measurement</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>valid بعد از سه فریم کامل و پایدار true شود</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>MEASUREMENT_WARMUP_FRAME_COUNT</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>MS-001..006</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>در انتظار برد</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="32" customHeight="1" s="4">
-      <c r="A5" s="8" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>REQ-M-002</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Measurement</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>فریم ناقص warm-up را reset کند</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>BSP ADC stable frame</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>MS-005, MS-018</t>
         </is>
       </c>
-      <c r="F5" s="8" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>در انتظار برد</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="32" customHeight="1" s="4">
-      <c r="A6" s="8" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>REQ-M-003</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Measurement</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>snapshot اتمیک و GetSnapshot(NULL)=false</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>measurement.c</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>MS-015, MS-016</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>در انتظار برد</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="32" customHeight="1" s="4">
-      <c r="A7" s="8" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>REQ-UI-001</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>snapshot invalid/NULL باعث safe-off و flag=false شود</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>ui_led.c</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>UI-023..025, UI-035</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>در انتظار برد</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="32" customHeight="1" s="4">
-      <c r="A8" s="8" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>REQ-UI-002</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Battery flag با 21000/21200 hysteresis و level پیوسته</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>UI_LOW_BATTERY...</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>UI_LOW_BATTERY_..</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>UI-027..030, UI-037</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>در انتظار برد</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="32" customHeight="1" s="4">
-      <c r="A9" s="8" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>REQ-BZ-001</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Buzzer</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>zero معتبر خاموش؛ ورودی نامعتبر -1 و Low</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>ui_buzzer.h</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>BZ-003..009</t>
         </is>
       </c>
-      <c r="F9" s="8" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>در انتظار برد</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="32" customHeight="1" s="4">
-      <c r="A10" s="8" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>REQ-BZ-002</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Buzzer</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>الگوی ON/gap/tail/nextCheck دقیق و non-blocking</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>ui_buzzer.c</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>BZ-001, BZ-010..022</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>در انتظار برد</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="32" customHeight="1" s="4">
-      <c r="A11" s="8" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>REQ-CO-001</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Changeover</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>invalid قبل از state/fault/pin و timerها reset شوند</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>changeover.c</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>CO-001..003, CO-017</t>
         </is>
       </c>
-      <c r="F11" s="8" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>در انتظار برد</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="32" customHeight="1" s="4">
-      <c r="A12" s="8" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>REQ-CO-002</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Changeover</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>fault معتبر → FAULT بدون تغییر pin</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>fault_mask</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>CO-004, CO-005, CO-018</t>
         </is>
       </c>
-      <c r="F12" s="8" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>نیازمند injection</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="32" customHeight="1" s="4">
-      <c r="A13" s="8" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>REQ-CO-003</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Changeover</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>mapping BATTERY/INPUT و SAFE/INPUT درست باشد</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>changeover.c</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>CO-006..016</t>
         </is>
       </c>
-      <c r="F13" s="8" t="inlineStr">
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>در انتظار برد</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="32" customHeight="1" s="4">
-      <c r="A14" s="8" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>REQ-CO-004</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Changeover</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>cut گیت‌شده و مستقل هر دو 3000ms پیوسته</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>21000/20800/3000ms</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>CO-008..012</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>در انتظار برد</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="32" customHeight="1" s="4">
-      <c r="A15" s="8" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>REQ-CO-005</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>Changeover</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>reconnect با input و &gt;=21200 بعد از 3000ms</t>
-        </is>
-      </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>21200/3000ms</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>reconnect با input و ≥21200 بعد از 30s+3s</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>21200/30000ms/3000ms</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>CO-013..016</t>
         </is>
       </c>
-      <c r="F15" s="8" t="inlineStr">
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>در انتظار برد</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="32" customHeight="1" s="4">
-      <c r="A16" s="8" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>REQ-CO-006</t>
         </is>
       </c>
-      <c r="B16" s="8" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>فقط BSP_GPIO_PROTECT_BATTERY؛ PB5/PB7/HAL ممنوع</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>changeover.c</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>CO-019, CO-020</t>
         </is>
       </c>
-      <c r="F16" s="8" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>بازبینی کد + برد</t>
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>REQ-CO-007</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Changeover</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>بازیابی بدون برق شهر: ۱۰s سالمِ بی‌وقفه + 3s؛ قطع دوباره داخل ۶۰s = باتری ضعیف؛ پاک‌شدن حکم با ۱۰ دقیقه سالم یا ریست دستی</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>147..157 (weak) + 150/149/148</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>تست‌های سناریوی ۸</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>در انتظار برد</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>REQ-LOG-001</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Panel log</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>تاریخچهٔ وضعیت همیشه می‌نویسد (حتی بدون برد) و ردیف قطع/وصل برق شهر حداکثر ۲۵۰ms بعد می‌نشیند تا با خاموشی ناگهانی پنل از دست نرود</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>SIMPLE_LOG_MAINS_FLUSH_MS/ESP_LOG_MAINS_FLUSH_MS</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>تست‌های هاست لاگ</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>انجام شد (Host)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F16"/>
-  <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
+  <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="001F4E79"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" style="4" min="1" max="1"/>
-    <col width="18" customWidth="1" style="4" min="2" max="2"/>
-    <col width="48" customWidth="1" style="4" min="3" max="3"/>
-    <col width="50" customWidth="1" style="4" min="4" max="4"/>
-    <col width="62" customWidth="1" style="4" min="5" max="5"/>
-    <col width="42" customWidth="1" style="4" min="6" max="6"/>
-    <col width="26" customWidth="1" style="4" min="7" max="7"/>
-    <col width="18" customWidth="1" style="4" min="8" max="8"/>
-    <col width="34" customWidth="1" style="4" min="9" max="9"/>
-    <col width="24" customWidth="1" style="4" min="10" max="10"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" s="4">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>Test Cases — سناریوهای اجرایی</t>
-        </is>
-      </c>
-      <c r="B1" s="6" t="n"/>
-      <c r="C1" s="6" t="n"/>
-      <c r="D1" s="6" t="n"/>
-      <c r="E1" s="6" t="n"/>
-      <c r="F1" s="6" t="n"/>
-      <c r="G1" s="6" t="n"/>
-      <c r="H1" s="6" t="n"/>
-      <c r="I1" s="6" t="n"/>
-      <c r="J1" s="5" t="n"/>
-    </row>
-    <row r="2" ht="42" customHeight="1" s="4">
-      <c r="A2" s="8" t="inlineStr">
-        <is>
-          <t>تست‌های هر ماژول فقط در فایل ولیدیشن همان ماژول است (پوشهٔ Firmware/Modules) و اینجا تکرار نمی‌شود؛ این شیت فقط تست‌های سطح سیستم را نگه می‌دارد. روش را اجرا کن و نتیجهٔ واقعی و مدرک را همین‌جا ثبت کن.</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="n"/>
-      <c r="C2" s="6" t="n"/>
-      <c r="D2" s="6" t="n"/>
-      <c r="E2" s="6" t="n"/>
-      <c r="F2" s="6" t="n"/>
-      <c r="G2" s="6" t="n"/>
-      <c r="H2" s="6" t="n"/>
-      <c r="I2" s="6" t="n"/>
-      <c r="J2" s="5" t="n"/>
-    </row>
-    <row r="3" ht="42" customHeight="1" s="4">
-      <c r="A3" s="9" t="inlineStr">
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Test Cases — سناریوهای اجرایی سطح سیستم</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>تست‌های هر ماژول فقط در فایل ولیدیشن همان ماژول است (پوشهٔ Firmware/Modules) و اینجا تکرار نمی‌شود؛ این شیت فقط تست‌های سطح سیستم را نگه می‌دارد.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Area</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Setup / input</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>روش اجرا</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
-        <is>
-          <t>نتیجه مورد انتظار</t>
-        </is>
-      </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>نتیجهٔ مورد انتظار</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>معیار قبولی</t>
         </is>
       </c>
-      <c r="G3" s="9" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>مرجع جزئیات</t>
         </is>
       </c>
-      <c r="H3" s="9" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="I3" s="9" t="inlineStr">
-        <is>
-          <t>نتیجه واقعی</t>
-        </is>
-      </c>
-      <c r="J3" s="9" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>نتیجهٔ واقعی</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>مدرک</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="54" customHeight="1" s="4">
-      <c r="A4" s="8" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>SYS-001</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Startup</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Build فعال با UI/Measurement/Changeover/Fault=1</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Clean build، پروگرام، Reset</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>بدون HardFault؛ taskهای فعال start شوند</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t>Reset و taskها پایدار</t>
-        </is>
-      </c>
-      <c r="G4" s="8" t="inlineStr">
-        <is>
-          <t>چهار Workbook، راهنما</t>
-        </is>
-      </c>
-      <c r="H4" s="8" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Reset و اجرای پیوسته</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>در انتظار</t>
         </is>
       </c>
-      <c r="I4" s="0" t="inlineStr"/>
-      <c r="J4" s="0" t="inlineStr"/>
-    </row>
-    <row r="5" ht="54" customHeight="1" s="4">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="I4" s="5" t="inlineStr"/>
+      <c r="J4" s="5" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>SYS-002</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>State log</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>پنل با/بدون برد؛ قطع و وصل شارژر</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>تغییر حالت‌ها و نگاه به تاریخچهٔ وضعیت</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>ردیف بوت، ردیف قطع/وصل برق شهر (≤۲۵۰ms)، ضربان ۶ساعته</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>هیچ تغییری بدون ردیف نماند</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>تست‌های هاست لاگ</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>انجام شد (Host)</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr"/>
+      <c r="J5" s="4" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>BZ-001</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Buzzer</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>period=10000,duty=10,count=1,gap=0</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>15s با scope/timer</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>ON=1000 و tail=9000</t>
         </is>
       </c>
-      <c r="F5" s="8" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>انحراف مجاز طبق Excel</t>
         </is>
       </c>
-      <c r="G5" s="8" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>Buzzer BZ-001</t>
         </is>
       </c>
-      <c r="H5" s="8" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>در انتظار</t>
         </is>
       </c>
-      <c r="I5" s="0" t="inlineStr"/>
-      <c r="J5" s="0" t="inlineStr"/>
-    </row>
-    <row r="6" ht="54" customHeight="1" s="4">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr"/>
+      <c r="J6" s="5" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>BZ-003</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Buzzer</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>period=10000,duty=0</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>الگو را اجرا کن</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>Low و return=0</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>خاموشی امن</t>
         </is>
       </c>
-      <c r="G6" s="8" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>Buzzer BZ-003</t>
         </is>
       </c>
-      <c r="H6" s="8" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>در انتظار</t>
         </is>
       </c>
-      <c r="I6" s="0" t="inlineStr"/>
-      <c r="J6" s="0" t="inlineStr"/>
-    </row>
-    <row r="7" ht="54" customHeight="1" s="4">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr"/>
+      <c r="J7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>BZ-006</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Buzzer</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>period=500,duty=50,count=1</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>الگو را اجرا کن</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Low و return=-1</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>نامعتبر رد شود</t>
         </is>
       </c>
-      <c r="G7" s="8" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>Buzzer BZ-006</t>
         </is>
       </c>
-      <c r="H7" s="8" t="inlineStr">
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>در انتظار</t>
         </is>
       </c>
-      <c r="I7" s="0" t="inlineStr"/>
-      <c r="J7" s="0" t="inlineStr"/>
-    </row>
-    <row r="8" ht="54" customHeight="1" s="4">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="I8" s="5" t="inlineStr"/>
+      <c r="J8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>BZ-017</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Buzzer</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>الگوی non-blocking فعال</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>Measurement را همزمان مانیتور کن</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>Measurement هر 10ms ادامه یابد</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>task قفل نشود</t>
         </is>
       </c>
-      <c r="G8" s="8" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>Buzzer BZ-017</t>
         </is>
       </c>
-      <c r="H8" s="8" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>در انتظار</t>
         </is>
       </c>
-      <c r="I8" s="0" t="inlineStr"/>
-      <c r="J8" s="0" t="inlineStr"/>
-    </row>
-    <row r="9" ht="54" customHeight="1" s="4">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr"/>
+      <c r="J9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>SAFE-001</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>GPIO</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>برد در تمام سناریوها</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>PB5/PB7/PB11 را مانیتور کن</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>فقط PB11 در cut/reconnect تغییر کند</t>
         </is>
       </c>
-      <c r="F9" s="8" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>PB5/PB7 بدون تغییر</t>
         </is>
       </c>
-      <c r="G9" s="8" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>CO-019/020</t>
         </is>
       </c>
-      <c r="H9" s="8" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>در انتظار</t>
         </is>
       </c>
-      <c r="I9" s="0" t="inlineStr"/>
-      <c r="J9" s="0" t="inlineStr"/>
-    </row>
-    <row r="10" ht="54" customHeight="1" s="4"/>
-    <row r="11" ht="54" customHeight="1" s="4"/>
-    <row r="12" ht="54" customHeight="1" s="4"/>
-    <row r="13" ht="54" customHeight="1" s="4"/>
-    <row r="14" ht="54" customHeight="1" s="4"/>
-    <row r="15" ht="54" customHeight="1" s="4"/>
-    <row r="16" ht="54" customHeight="1" s="4"/>
-    <row r="17" ht="54" customHeight="1" s="4"/>
-    <row r="18" ht="54" customHeight="1" s="4"/>
-    <row r="19" ht="54" customHeight="1" s="4"/>
-    <row r="20" ht="54" customHeight="1" s="4"/>
-    <row r="21" ht="54" customHeight="1" s="4"/>
-    <row r="22" ht="54" customHeight="1" s="4"/>
-    <row r="23" ht="54" customHeight="1" s="4"/>
-    <row r="24" ht="54" customHeight="1" s="4"/>
-    <row r="25" ht="54" customHeight="1" s="4"/>
-    <row r="26" ht="54" customHeight="1" s="4"/>
-    <row r="27" ht="54" customHeight="1" s="4"/>
-    <row r="28" ht="54" customHeight="1" s="4"/>
-    <row r="29" ht="54" customHeight="1" s="4"/>
-    <row r="30" ht="54" customHeight="1" s="4"/>
-    <row r="31" ht="54" customHeight="1" s="4"/>
-    <row r="32" ht="54" customHeight="1" s="4"/>
+      <c r="I10" s="5" t="inlineStr"/>
+      <c r="J10" s="5" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:J32"/>
-  <mergeCells count="2">
+  <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00BF8F00"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" style="4" min="1" max="1"/>
-    <col width="34" customWidth="1" style="4" min="2" max="2"/>
-    <col width="48" customWidth="1" style="4" min="3" max="3"/>
-    <col width="18" customWidth="1" style="4" min="4" max="4"/>
-    <col width="42" customWidth="1" style="4" min="5" max="5"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" s="4">
-      <c r="A1" s="7" t="inlineStr">
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Coverage — پوشش الزامات با تست‌ها</t>
         </is>
       </c>
-      <c r="B1" s="6" t="n"/>
-      <c r="C1" s="6" t="n"/>
-      <c r="D1" s="6" t="n"/>
-      <c r="E1" s="5" t="n"/>
-    </row>
-    <row r="2" ht="42" customHeight="1" s="4">
-      <c r="A2" s="8" t="inlineStr">
-        <is>
-          <t>این صفحه برای پیدا کردن سناریوهای جاافتاده است؛ GAP نباید بی‌توضیح باقی بماند.</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="n"/>
-      <c r="C2" s="6" t="n"/>
-      <c r="D2" s="6" t="n"/>
-      <c r="E2" s="5" t="n"/>
-    </row>
-    <row r="3" ht="42" customHeight="1" s="4">
-      <c r="A3" s="9" t="inlineStr">
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Covered by tests</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Expected evidence</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Gap / action</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="32" customHeight="1" s="4">
-      <c r="A4" s="8" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Measurement warm-up</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>MS-001..005</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Live snapshot + timing</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>در انتظار</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>سه فریم کامل و فریم ناپایدار</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="32" customHeight="1" s="4">
-      <c r="A5" s="8" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Measurement conversion</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>MS-004, MS-007, MS-020, MS-021</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>DMM + raw counts + live values</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>در انتظار</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>مقادیر واقعی ثبت شود</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="32" customHeight="1" s="4">
-      <c r="A6" s="8" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>UI safe-off</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>UI-023, UI-024</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>LED/Buzzer voltage and flag</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>در انتظار</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>NULL/invalid تزریق شود</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="32" customHeight="1" s="4">
-      <c r="A7" s="8" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>UI hysteresis</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>UI-027, UI-029</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>flag trace</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>در انتظار</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>21000/21200 تست شود</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="32" customHeight="1" s="4">
-      <c r="A8" s="8" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Buzzer timing</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>BZ-001, BZ-010..017</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>scope/timer CSV</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>در انتظار</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>مدت ON/gap/tail ثبت شود</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="32" customHeight="1" s="4">
-      <c r="A9" s="8" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Changeover mapping</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>CO-006, CO-007</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>state + PB11</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>در انتظار</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>BATTERY/INPUT ثبت شود</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="32" customHeight="1" s="4">
-      <c r="A10" s="8" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Changeover cut</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>CO-008..012</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>time + PB11 + state</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>در انتظار</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>2500/3000ms و مرزها</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="32" customHeight="1" s="4">
-      <c r="A11" s="8" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Changeover reconnect</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>CO-013..016</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>time + PB11 + state</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>در انتظار</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>21200 و کمتر از 3s</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="32" customHeight="1" s="4">
-      <c r="A12" s="8" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Weak-battery recovery</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>سناریوی ۸</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>time + face + one retry</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>در انتظار</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>10s hold، 60s cycle guard، 10min clear</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>State log completeness</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>SYS-002 + تست‌های هاست</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>فایل‌های روزانه + CSV</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>انجام شد (Host)</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>روی برد واقعی تکرار شود</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Fault valid</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>FL-001</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>fault injection + state/pin</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>نیازمند injection</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>Protection خاموش است</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="32" customHeight="1" s="4">
-      <c r="A13" s="8" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Fault invalid</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>FL-002</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>fault injection + preserved state/pin</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>نیازمند injection</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>invalid باید قبل از fault باشد</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="32" customHeight="1" s="4">
-      <c r="A14" s="8" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>GPIO restriction</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>SAFE-001</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>scope/logic analyzer</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>در انتظار</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>PB5/PB7 بدون تغییر</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:E14"/>
-  <mergeCells count="2">
-    <mergeCell ref="A2:E2"/>
+  <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
-  <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00BF8F00"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" style="4" min="1" max="1"/>
-    <col width="20" customWidth="1" style="4" min="2" max="2"/>
-    <col width="46" customWidth="1" style="4" min="3" max="3"/>
-    <col width="28" customWidth="1" style="4" min="4" max="4"/>
-    <col width="28" customWidth="1" style="4" min="5" max="5"/>
-    <col width="24" customWidth="1" style="4" min="6" max="6"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" s="4">
-      <c r="A1" s="7" t="inlineStr">
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Signals — سیگنال‌ها و مالکیت داده</t>
         </is>
       </c>
-      <c r="B1" s="6" t="n"/>
-      <c r="C1" s="6" t="n"/>
-      <c r="D1" s="6" t="n"/>
-      <c r="E1" s="6" t="n"/>
-      <c r="F1" s="5" t="n"/>
-    </row>
-    <row r="2" ht="42" customHeight="1" s="4">
-      <c r="A2" s="8" t="inlineStr">
-        <is>
-          <t>مالک هر سیگنال مشخص است؛ ماژول دیگر نباید state داخلی مالک را مستقیم تغییر دهد.</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="n"/>
-      <c r="C2" s="6" t="n"/>
-      <c r="D2" s="6" t="n"/>
-      <c r="E2" s="6" t="n"/>
-      <c r="F2" s="5" t="n"/>
-    </row>
-    <row r="3" ht="42" customHeight="1" s="4">
-      <c r="A3" s="9" t="inlineStr">
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Signal / variable</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Meaning</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Readers</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Writer / source</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Safe/default</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="32" customHeight="1" s="4">
-      <c r="A4" s="8" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>measurement_snapshot_t</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Measurement</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>داده اتمیک ADC و input</t>
-        </is>
-      </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>دادهٔ اتمیک ADC و input</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>UI, Changeover, Protection, Charger, McuPowerPath</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>Measurement task</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>valid=false</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="32" customHeight="1" s="4">
-      <c r="A5" s="8" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>snapshot.valid</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Measurement</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>آماده‌بودن داده بعد از warm-up</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>UI, Changeover, Charger, Fault</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>Measurement</t>
         </is>
       </c>
-      <c r="F5" s="8" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="32" customHeight="1" s="4">
-      <c r="A6" s="8" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>snapshot.v_bat24_mv</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Measurement</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>ولتاژ باتری 24V</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>UI, Changeover</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Measurement</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="32" customHeight="1" s="4">
-      <c r="A7" s="8" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>snapshot.input_present</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Measurement</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>حضور ورودی اصلی</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>UI, Changeover</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>BSP/Measurement</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="32" customHeight="1" s="4">
-      <c r="A8" s="8" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>BOOL__G__UiBatteryAlarmIssued</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>آلارم باتری کم با hysteresis</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Changeover</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="32" customHeight="1" s="4">
-      <c r="A9" s="8" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>fault_mask</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Fault</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>خطاهای مشترک لچ‌شده</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>Changeover, Charger, UI, Comm</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Fault producers</t>
         </is>
       </c>
-      <c r="F9" s="8" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>FAULT_NONE</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="32" customHeight="1" s="4">
-      <c r="A10" s="8" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>BSP_GPIO_PROTECT_BATTERY</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>BSP/Changeover</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>PB11 منطقی حفاظت باتری</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>BSP</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>Changeover only</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>false = Safe High</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="32" customHeight="1" s="4">
-      <c r="A11" s="8" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>PB5/PB7</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>BSP</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>پایه‌های خارج از مالکیت Changeover</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>هیچ‌کدام در Changeover</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>ماژول‌های مجاز خودشان</t>
         </is>
       </c>
-      <c r="F11" s="8" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>بدون تغییر</t>
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>CH_PD (ESP power)</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>EspLink</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>تغذیهٔ ماژول وای‌فای با سیاست صرفه‌جویی</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>EspLink_Power (با مهلت ۴۰۰ms برای آخرین فریم)</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>snapshot.values (کانال‌های جریان/نیم‌باتری)</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>Measurement</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>جریان شارژ فیلترشده (median-3 → میانگین-10، کلیدها در measurement.h) و ولتاژ نیم‌های 12V (مبنای قواعد قطع باتری 6V/7V)</t>
-        </is>
-      </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>Charger, Fault, UI</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="inlineStr">
-        <is>
-          <t>Measurement task</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>valid=false / 0</t>
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>تاریخچهٔ وضعیت (پنل)</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Panel (ESP)</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>ردیف‌های تغییر وضعیت روی LittleFS</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>کارت تاریخچه + دانلود CSV</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>OnFrame/Tick پنل</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>روز بدون ساعت</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:F11"/>
-  <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
+  <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00BF8F00"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" style="4" min="1" max="1"/>
-    <col width="28" customWidth="1" style="4" min="2" max="2"/>
-    <col width="42" customWidth="1" style="4" min="3" max="3"/>
-    <col width="24" customWidth="1" style="4" min="4" max="4"/>
-    <col width="52" customWidth="1" style="4" min="5" max="5"/>
-    <col width="24" customWidth="1" style="4" min="6" max="6"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" s="4">
-      <c r="A1" s="7" t="inlineStr">
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Faults — ماسک خطا و روش تزریق</t>
         </is>
       </c>
-      <c r="B1" s="6" t="n"/>
-      <c r="C1" s="6" t="n"/>
-      <c r="D1" s="6" t="n"/>
-      <c r="E1" s="6" t="n"/>
-      <c r="F1" s="5" t="n"/>
-    </row>
-    <row r="2" ht="42" customHeight="1" s="4">
-      <c r="A2" s="8" t="inlineStr">
-        <is>
-          <t>Fault mask مرکزی است؛ با Protection خاموش، تست Fault نیازمند injection است.</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="n"/>
-      <c r="C2" s="6" t="n"/>
-      <c r="D2" s="6" t="n"/>
-      <c r="E2" s="6" t="n"/>
-      <c r="F2" s="5" t="n"/>
-    </row>
-    <row r="3" ht="42" customHeight="1" s="4">
-      <c r="A3" s="9" t="inlineStr">
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Fault bit</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Intended producer</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Meaning</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Consumer</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Test method now</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Recovery</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="32" customHeight="1" s="4">
-      <c r="A4" s="8" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>FAULT_ADC</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Protection/Measurement</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>ADC/snapshot fault</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>Changeover</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>func__Fault_Set injection؛ Protection فعلاً off</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>Fault_Clear/test reset</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="32" customHeight="1" s="4">
-      <c r="A5" s="8" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>FAULT_OVERCURRENT_1</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Protection</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>جریان کانال 1 بیش از حد</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Changeover</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>injection؛ threshold کامل نشده</t>
         </is>
       </c>
-      <c r="F5" s="8" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>Fault_Clear</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="32" customHeight="1" s="4">
-      <c r="A6" s="8" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>FAULT_OVERCURRENT_2</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Protection</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>جریان کانال 2 بیش از حد</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Changeover</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>injection؛ threshold کامل نشده</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>Fault_Clear</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="32" customHeight="1" s="4">
-      <c r="A7" s="8" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>FAULT_LOW_BATTERY</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Protection/UI policy</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>خطای کم‌باتری ایمنی</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>Changeover</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>injection؛ UI flag جداست</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>Fault_Clear</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="32" customHeight="1" s="4">
-      <c r="A8" s="8" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>FAULT_JITTER_1</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Jitter</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>رویداد jitter خط 1</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Charger (JIT retry), Comm</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>روی برد: پالس LM393 → EXTI؛ Jitter فعال است (2026-09-22). در host: injection</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>Fault_Clear</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="32" customHeight="1" s="4">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>روی برد: پالس LM393 → EXTI؛ در host: injection</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>auto/retry</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>FAULT_JITTER_2</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Jitter</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>رویداد jitter خط 2</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>Charger (JIT retry), Comm</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
-        <is>
-          <t>روی برد: پالس LM393 → EXTI؛ Jitter فعال است (2026-09-22). در host: injection</t>
-        </is>
-      </c>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>Fault_Clear</t>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>روی برد: پالس LM393 → EXTI؛ در host: injection</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>auto/retry</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>FAULT_CHARGER_BAT_LOST</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Fault</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>قطع باتری: پمپ &gt;14.8V حین شارژ (150ms) یا هر نیم &lt;6V با ورودی سالم (1s)</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Charger, UI</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>تزریق/سیم‌کشی</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>باتری برگردد + 1s پایدار</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>FAULT_CHARGER_BAT_LOST</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>Fault</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>قطع باتری: پمپ &gt;FAULT_BAT_DISCONNECT_MV=14.8V حین شارژ (150ms) یا هر نیم &lt;FAULT_BAT_ABSENT_MV=6V با ورودی سالم (1s)</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>Charger (آینه به CHG_STATE_BAT_LOST و پارک PWM)</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr">
-        <is>
-          <t>host_test_charger.py قواعد rule-1/rule-2؛ روی برد: کشیدن سیم نیم/کل باتری</t>
-        </is>
-      </c>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>Clear توسط Fault: هر دو نیم ≥FAULT_BATTERY_BACK_MV=7V بدون پمپ برای 1s (هیسترزیس 1V عمدی)</t>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>FAULT_CHARGER_TECHNICAL</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Charger (scenario 7)</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>مسیر قدرت: duty&gt;200‰ با جریان صفر (و بالعکس)</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>UI, Panel</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>تزریق</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>خاموش/روشن تا ریست؛ قفل نهایی فقط با ریست برد</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:F9"/>
-  <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
+  <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00A6A6A6"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" style="4" min="1" max="1"/>
-    <col width="42" customWidth="1" style="4" min="2" max="2"/>
-    <col width="60" customWidth="1" style="4" min="3" max="3"/>
-    <col width="28" customWidth="1" style="4" min="4" max="4"/>
-    <col width="42" customWidth="1" style="4" min="5" max="5"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" s="4">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>Change Log — تاریخچه تغییرات</t>
-        </is>
-      </c>
-      <c r="B1" s="6" t="n"/>
-      <c r="C1" s="6" t="n"/>
-      <c r="D1" s="6" t="n"/>
-      <c r="E1" s="5" t="n"/>
-    </row>
-    <row r="2" ht="42" customHeight="1" s="4">
-      <c r="A2" s="8" t="inlineStr">
-        <is>
-          <t>تغییرات مستند این مرجع و مبنای firmware را ثبت کن.</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="n"/>
-      <c r="C2" s="6" t="n"/>
-      <c r="D2" s="6" t="n"/>
-      <c r="E2" s="5" t="n"/>
-    </row>
-    <row r="3" ht="42" customHeight="1" s="4">
-      <c r="A3" s="9" t="inlineStr">
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Change Log — تاریخچهٔ تغییرات</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Change</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Reason</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Source commit</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Validation</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="32" customHeight="1" s="4">
-      <c r="A4" s="8" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>ساخت مرجع Master State و Scenario</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>قابل‌فهم‌کردن stateها، transitionها و پوشش تست</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>b64d7ed base</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>این Workbook + draw.io</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="32" customHeight="1" s="4">
-      <c r="A5" s="8" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>وضعیت فعال‌سازی</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>UI/Measurement/Changeover/Fault برای build تستی فعال؛ Protection و ماژول‌های آینده خاموش</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>b64d7ed</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
-        <is>
-          <t>فلگ‌ها در modules_enable.h</t>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>فلگ‌ها در modules_config</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>ممیزی کامل برنامه (فیکس race در BspExti_TakeEvent، FAULT_ADC لحظه‌ای، حذف هوک تکراری ISR)؛ فیلترهای جریان median-3 → میانگین-10</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>هماهنگی با کد</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>تست‌های هاست</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>ممیزی کامل برنامه (فیکس race در BspExti_TakeEvent، FAULT_ADC لحظه‌ای، حذف هوک تکراری ISR)؛ فیلترهای جریان median-3 → میانگین-10 با کلید کامپایل؛ جداسازی آستانهٔ قطع باتری (تشخیص 6V / بازیابی 7V)؛ به‌روزرسانی برگه‌های راهنما/Signals/Faults</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>دستور کاربر: چک کامل برنامه، اصلاح ایرادها و آپدیت مدارک</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>arena/01a0c744-changeover (این commit)</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>check_firmware_syntax PASS؛ host_test_charger 23/23؛ check_ai_rules فقط [17] شناخته‌شده</t>
-        </is>
-      </c>
-    </row>
-    <row r="7"/>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>بازسازی هر دو Workbook (State.xlsx و همین فایل) از کد فعلی با ابزار tools/make_state_reference_xlsx.py: جدول چراغ‌ها/بوق، پنجرهٔ ورودی ۲۱..۲۸، قواعد وصل مجدد بدون برق شهر (ST-011..013) و الزام کامل‌بودن لاگ (REQ-LOG-001)</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>دستور کاربر: «اکسل‌ها را با کد فعلی به‌روز کن»</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>v1.108</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>تست‌های هاست + تولید ابزار</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:E5"/>
-  <mergeCells count="2">
-    <mergeCell ref="A2:E2"/>
+  <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
-  <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
v1.109: battery state in every log row (batt_pct column + mode + watts) + every rise in discharge records a row; fix preview self-test hang
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Documentation/System_State_Scenarios.xlsx
+++ b/Documentation/System_State_Scenarios.xlsx
@@ -2028,12 +2028,12 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>تاریخچهٔ وضعیت همیشه می‌نویسد (حتی بدون برد) و ردیف قطع/وصل برق شهر حداکثر ۲۵۰ms بعد می‌نشیند تا با خاموشی ناگهانی پنل از دست نرود</t>
+          <t>تاریخچهٔ وضعیت همیشه می‌نویسد (حتی بدون برد)، ردیف قطع/وصل برق شهر حداکثر ۲۵۰ms بعد می‌نشیند، هر خط وضعیت باتری (درصد/حالت/وات) را می‌گوید و در دشارژ هر بالا آمدنِ پک (پلهٔ ۲۰۰ میلی‌ولتی) ردیف خودش را می‌نویسد</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>SIMPLE_LOG_MAINS_FLUSH_MS/ESP_LOG_MAINS_FLUSH_MS</t>
+          <t>SIMPLE_LOG_MAINS_FLUSH_MS/ESP_LOG_MAINS_FLUSH_MS + ستون batt_pct + قانون VSTEP صعودی</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">

</xml_diff>